<commit_message>
Carga de cafe de Consum completa: Chocolate fuerte y Leche al cacao al precio de chocolate, y fuera las dos maquinas con cafe distinto
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019AhsUdeCJveFgyWPkWGnqu
</commit_message>
<xml_diff>
--- a/carga/tarifa_consum_cafe.xlsx
+++ b/carga/tarifa_consum_cafe.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -442,11 +442,11 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,119 +459,83 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Precios de la tarifa de Gonzalo del 27-07-2026. El precio va por selección, no por marca de café.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+          <t>Precios de la tarifa del 27-07-2026. El precio va por selección, no por marca de café.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Excluidas 26CE5204 (Cox) y 26CE5209 (Toledo): llevan café distinto y hay que revisarlas aparte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Cod. artículo</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Selección</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Gama</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Precio efectivo</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Precio tarjeta privada</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Precio tarjeta crédito</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Canales afectados</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Canales</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Máquinas</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Precio actual mín</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Precio actual máx</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Línea en la tarifa de Gonzalo</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>R01</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Café solo normal</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G5" t="n">
-        <v>17</v>
-      </c>
-      <c r="H5" t="n">
-        <v>17</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>CAFE ESPRESSO CORTO</t>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Referencia en la tarifa del 27-07-2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>R02</t>
+          <t>R01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Café largo normal</t>
+          <t>Café solo normal</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -589,32 +553,32 @@
         <v>0.4</v>
       </c>
       <c r="G6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>0.45</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.8</v>
+        <v>0.45</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>CAFÉ ESPRESSO BAR LARGO</t>
+          <t>CAFE ESPRESSO CORTO</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>R03</t>
+          <t>R02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Café cortado normal</t>
+          <t>Café largo normal</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -632,32 +596,32 @@
         <v>0.4</v>
       </c>
       <c r="G7" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H7" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>0.45</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>1</v>
+        <v>0.45</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>CAFÉ ESPRESSO BAR CORTADO</t>
+          <t>CAFÉ ESPRESSO BAR LARGO</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>R04</t>
+          <t>R03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Café con leche normal</t>
+          <t>Café cortado normal</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -675,32 +639,32 @@
         <v>0.4</v>
       </c>
       <c r="G8" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H8" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0.45</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>1</v>
+        <v>0.45</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>CAFÉ ESPRESSO BAR CON LECHE</t>
+          <t>CAFÉ ESPRESSO BAR CORTADO</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>R05</t>
+          <t>R04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cappuccino normal</t>
+          <t>Café con leche normal</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -712,38 +676,38 @@
         <v>0.45</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="G9" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H9" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>CAFÉ ESPRESSO BAR CAPUCHINO</t>
+          <t>CAFÉ ESPRESSO BAR CON LECHE</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>R06</t>
+          <t>R05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Leche manchada normal</t>
+          <t>Cappuccino normal</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -755,10 +719,10 @@
         <v>0.45</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="G10" t="n">
         <v>16</v>
@@ -767,69 +731,69 @@
         <v>16</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>CAFÉ ESPRESSO BAR LECHE MANCHADA</t>
+          <t>CAFÉ ESPRESSO BAR CAPUCHINO</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>R10</t>
+          <t>R06</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Café solo premium</t>
+          <t>Leche manchada normal</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.55</v>
+        <v>0.4</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.55</v>
+        <v>0.4</v>
       </c>
       <c r="G11" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H11" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>CAFE SALZILLO CORTO</t>
+          <t>CAFÉ ESPRESSO BAR LECHE MANCHADA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Café largo premium</t>
+          <t>Café solo premium</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -847,32 +811,32 @@
         <v>0.55</v>
       </c>
       <c r="G12" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="H12" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>0.6</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>CAFÉ SALZILLO LARGO</t>
+          <t>CAFE SALZILLO CORTO</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Café cortado premium</t>
+          <t>Café largo premium</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -890,32 +854,32 @@
         <v>0.55</v>
       </c>
       <c r="G13" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="H13" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>0.6</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>CAFÉ SALZILLO CORTADO</t>
+          <t>CAFÉ SALZILLO LARGO</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Café con leche premium</t>
+          <t>Café cortado premium</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -933,32 +897,32 @@
         <v>0.55</v>
       </c>
       <c r="G14" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="H14" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>0.6</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>CAFÉ SALZILLO CON LECHE</t>
+          <t>CAFÉ SALZILLO CORTADO</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cappuccino premium</t>
+          <t>Café con leche premium</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -967,41 +931,41 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="G15" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H15" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>CAFÉ SALZILLO CAPUCHINO</t>
+          <t>CAFÉ SALZILLO CON LECHE</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>R13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Leche manchada premium</t>
+          <t>Cappuccino premium</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1010,84 +974,84 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="G16" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H16" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>CAFÉ SALZILLO LECHE MANCAHADA</t>
+          <t>CAFÉ SALZILLO CAPUCHINO</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>R22</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Café solo descafeinado</t>
+          <t>Leche manchada premium</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Descafeinado</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0.45</v>
+        <v>0.6</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.4</v>
+        <v>0.55</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>0.4</v>
+        <v>0.55</v>
       </c>
       <c r="G17" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H17" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>DESCAFEINADO CORTO</t>
+          <t>CAFÉ SALZILLO LECHE MANCAHADA</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>R23</t>
+          <t>R22</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Café largo descafeinado</t>
+          <t>Café solo descafeinado</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1105,32 +1069,32 @@
         <v>0.4</v>
       </c>
       <c r="G18" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H18" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>0.45</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>DESCAFEINADO LARGO</t>
+          <t>DESCAFEINADO CORTO</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>R36</t>
+          <t>R23</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Café cortado descafeinado</t>
+          <t>Café largo descafeinado</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1148,32 +1112,32 @@
         <v>0.4</v>
       </c>
       <c r="G19" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H19" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>0.45</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>DESCAFEINADO CORTADO</t>
+          <t>DESCAFEINADO LARGO</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>R17</t>
+          <t>R36</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Café con leche descafeinado</t>
+          <t>Café cortado descafeinado</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1191,32 +1155,32 @@
         <v>0.4</v>
       </c>
       <c r="G20" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H20" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>1</v>
+        <v>0.45</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>DESCAFEINADO CON LECHE</t>
+          <t>DESCAFEINADO CORTADO</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>R27</t>
+          <t>R17</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cappuccino descafeinado</t>
+          <t>Café con leche descafeinado</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1228,10 +1192,10 @@
         <v>0.45</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="G21" t="n">
         <v>16</v>
@@ -1240,26 +1204,26 @@
         <v>16</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>DESCAFEINADO CAPUCHINO</t>
+          <t>DESCAFEINADO CON LECHE</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>R26</t>
+          <t>R27</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Leche manchada descafeinada</t>
+          <t>Cappuccino descafeinado</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1271,16 +1235,16 @@
         <v>0.45</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="G22" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="H22" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>0</v>
@@ -1290,24 +1254,24 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>LECHE MANCHADA DESCAFEINADA</t>
+          <t>DESCAFEINADO CAPUCHINO</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>R34</t>
+          <t>R26</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Leche</t>
+          <t>Leche manchada descafeinada</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Descafeinado</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1320,32 +1284,32 @@
         <v>0.4</v>
       </c>
       <c r="G23" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="H23" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>LECHE</t>
+          <t>LECHE MANCHADA DESCAFEINADA</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>R07</t>
+          <t>R34</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Chocolate</t>
+          <t>Leche</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1363,32 +1327,32 @@
         <v>0.4</v>
       </c>
       <c r="G24" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H24" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>CHOCOLATE</t>
+          <t>LECHE</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>R30</t>
+          <t>R07</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Chocolate con leche</t>
+          <t>Chocolate</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1406,32 +1370,32 @@
         <v>0.4</v>
       </c>
       <c r="G25" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H25" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>0.45</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>CHOCOLATE CON LECHE</t>
+          <t>CHOCOLATE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>R28</t>
+          <t>R30</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cappuccino vainilla</t>
+          <t>Chocolate con leche</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1440,19 +1404,19 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.55</v>
+        <v>0.45</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G26" t="n">
         <v>17</v>
       </c>
       <c r="H26" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>0</v>
@@ -1462,19 +1426,19 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>CAFE PREPARADO CAPUCCINO VAINILLA 1KG</t>
+          <t>CHOCOLATE CON LECHE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R44</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Cappuccino avellana</t>
+          <t>Chocolate fuerte</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1483,41 +1447,41 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G27" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="H27" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>CAFE PREPARADO CAPUCCINO AVELLANA 1KG</t>
+          <t>CHOCOLATE (precio de chocolate, confirmado)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>R44</t>
+          <t>R108</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Chocolate fuerte</t>
+          <t>Leche al cacao</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1526,13 +1490,13 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v/>
+        <v>0.45</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="G28" t="n">
         <v>5</v>
@@ -1548,19 +1512,19 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>SIN EQUIVALENTE — pendiente de Gonzalo</t>
+          <t>CHOCOLATE / LECHE (mismo precio en ambas)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>R108</t>
+          <t>R28</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Leche al cacao</t>
+          <t>Cappuccino vainilla</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1569,29 +1533,72 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v/>
+        <v>0.55</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v/>
+        <v>0.5</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v/>
+        <v>0.5</v>
       </c>
       <c r="G29" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="H29" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="I29" s="3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J29" s="3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>CAFE PREPARADO CAPUCCINO VAINILLA 1KG</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>R29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Cappuccino avellana</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G30" t="n">
+        <v>15</v>
+      </c>
+      <c r="H30" t="n">
+        <v>15</v>
+      </c>
+      <c r="I30" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>SIN EQUIVALENTE — pendiente de Gonzalo</t>
+      <c r="J30" s="3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>CAFE PREPARADO CAPUCCINO AVELLANA 1KG</t>
         </is>
       </c>
     </row>

</xml_diff>